<commit_message>
fix: switch header cells to place study info on left and logo on right
</commit_message>
<xml_diff>
--- a/templates/GCPS_DMF_012.8_A-CValidation Check QC Form.xlsx
+++ b/templates/GCPS_DMF_012.8_A-CValidation Check QC Form.xlsx
@@ -1869,11 +1869,11 @@
   <ns0:pageMargins left="0.23622047244094491" right="0.23622047244094491" top="1.08" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <ns0:pageSetup paperSize="9" scale="80" pageOrder="overThenDown" orientation="landscape" ns4:id="rId1"/>
   <ns0:headerFooter>
-    <ns0:oddHeader>&amp;L&amp;G&amp;C&amp;"Arial"&amp;16Validation Check QC Form
+    <ns0:oddHeader>&amp;L&amp;"Arial"&amp;10Study Code: &lt;Code&gt;
+System: QCTMS LC&amp;C&amp;"Arial"&amp;16Validation Check QC Form
 &amp;"Arial"&amp;14QCTMS LC
 &amp;"Arial"&amp;11Version No.: &lt;X.X&gt;
-&amp;"Arial"&amp;11Version Date: &lt;DD/MMM/YYYY&gt;&amp;R&amp;"Arial"&amp;10Study Code: &lt;Code&gt;
-System: QCTMS LC</ns0:oddHeader>
+&amp;"Arial"&amp;11Version Date: &lt;DD/MMM/YYYY&gt;&amp;R&amp;G</ns0:oddHeader>
     <ns0:oddFooter>&amp;L&amp;"Arial,Standard"GCPS_DMF_012.8_A&amp;C&amp;"Arial,Standard"Effective Date: 16/DEC/2024&amp;R&amp;"Arial,Standard"Page &amp;P of &amp;N</ns0:oddFooter>
   </ns0:headerFooter>
   <ns0:legacyDrawingHF ns4:id="rId2"/>
@@ -2293,11 +2293,11 @@
   <ns0:pageMargins left="0.23622047244094491" right="0.23622047244094491" top="1.06" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <ns0:pageSetup paperSize="9" scale="80" pageOrder="overThenDown" orientation="landscape" ns4:id="rId1"/>
   <ns0:headerFooter>
-    <ns0:oddHeader>&amp;L&amp;G&amp;C&amp;"Arial"&amp;16Validation Check QC Form
+    <ns0:oddHeader>&amp;L&amp;"Arial"&amp;10Study Code: &lt;Code&gt;
+System: Castor&amp;C&amp;"Arial"&amp;16Validation Check QC Form
 &amp;"Arial"&amp;14Castor
 &amp;"Arial"&amp;11Version No.: &lt;X.X&gt;
-&amp;"Arial"&amp;11Version Date: &lt;DD/MMM/YYYY&gt;&amp;R&amp;"Arial"&amp;10Study Code: &lt;Code&gt;
-System: Castor</ns0:oddHeader>
+&amp;"Arial"&amp;11Version Date: &lt;DD/MMM/YYYY&gt;&amp;R&amp;G</ns0:oddHeader>
     <ns0:oddFooter>&amp;L&amp;"Arial,Standard"GCPS_DMF_012.8_B&amp;C&amp;"Arial,Standard"Effective Date: 16/DEC/2024&amp;R&amp;"Arial,Standard"Page &amp;P of &amp;N</ns0:oddFooter>
   </ns0:headerFooter>
   <ns0:legacyDrawingHF ns4:id="rId2"/>
@@ -2387,11 +2387,11 @@
   <ns0:pageMargins left="0.23622047244094446" right="0.23622047244094446" top="1.0599999999999998" bottom="0.74803149606299169" header="0.31496062992125973" footer="0.31496062992125973"/>
   <ns0:pageSetup paperSize="9" scale="80" orientation="landscape" ns4:id="rId1"/>
   <ns0:headerFooter>
-    <ns0:oddHeader>&amp;L&amp;G&amp;C&amp;"Arial"&amp;16Validation Check QC Form
+    <ns0:oddHeader>&amp;L&amp;"Arial"&amp;10Study Code: &lt;Code&gt;
+System: Viedoc&amp;C&amp;"Arial"&amp;16Validation Check QC Form
 &amp;"Arial"&amp;14Data Checks
 &amp;"Arial"&amp;11Version No.: &lt;X.X&gt;
-&amp;"Arial"&amp;11Version Date: &lt;DD/MMM/YYYY&gt;&amp;R&amp;"Arial"&amp;10Study Code: &lt;Code&gt;
-System: Viedoc</ns0:oddHeader>
+&amp;"Arial"&amp;11Version Date: &lt;DD/MMM/YYYY&gt;&amp;R&amp;G</ns0:oddHeader>
     <ns0:oddFooter>&amp;L&amp;"Arial,Standard"GCPS_DMF_012.8_C1&amp;C&amp;"Arial,Standard"Effective Date: 16/DEC/2024&amp;R&amp;"Arial,Standard"Page &amp;P of &amp;N</ns0:oddFooter>
   </ns0:headerFooter>
   <ns0:legacyDrawingHF ns4:id="rId2"/>
@@ -2493,11 +2493,11 @@
   <ns0:pageMargins left="0.23622047244094446" right="0.23622047244094446" top="1.0599999999999998" bottom="0.74803149606299169" header="0.31496062992125973" footer="0.31496062992125973"/>
   <ns0:pageSetup paperSize="9" scale="80" orientation="landscape" ns4:id="rId1"/>
   <ns0:headerFooter>
-    <ns0:oddHeader>&amp;L&amp;G&amp;C&amp;"Arial"&amp;16Validation Check QC Form
+    <ns0:oddHeader>&amp;L&amp;"Arial"&amp;10Study Code: &lt;Code&gt;
+System: Viedoc&amp;C&amp;"Arial"&amp;16Validation Check QC Form
 &amp;"Arial"&amp;14Alerts
 &amp;"Arial"&amp;11Version No.: &lt;X.X&gt;
-&amp;"Arial"&amp;11Version Date: &lt;DD/MMM/YYYY&gt;&amp;R&amp;"Arial"&amp;10Study Code: &lt;Code&gt;
-System: Viedoc</ns0:oddHeader>
+&amp;"Arial"&amp;11Version Date: &lt;DD/MMM/YYYY&gt;&amp;R&amp;G</ns0:oddHeader>
     <ns0:oddFooter>&amp;L&amp;"Arial,Standard"GCPS_DMF_012.8_C2&amp;C&amp;"Arial,Standard"Effective Date: 16/DEC/2024&amp;R&amp;"Arial,Standard"Page &amp;P of &amp;N</ns0:oddFooter>
   </ns0:headerFooter>
   <ns0:legacyDrawingHF ns4:id="rId2"/>
@@ -3595,11 +3595,11 @@
   <ns0:pageMargins left="0.23622047244094491" right="0.23622047244094491" top="1.0733333333333333" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <ns0:pageSetup paperSize="9" scale="80" pageOrder="overThenDown" orientation="landscape" ns4:id="rId1"/>
   <ns0:headerFooter>
-    <ns0:oddHeader>&amp;L&amp;G&amp;C&amp;"Arial"&amp;16Validation Check QC Form
+    <ns0:oddHeader>&amp;L&amp;"Arial"&amp;10Study Code: &lt;Code&gt;
+System: &lt;System&gt;&amp;C&amp;"Arial"&amp;16Validation Check QC Form
 &amp;"Arial"&amp;14New
 &amp;"Arial"&amp;11Version No.: &lt;X.X&gt;
-&amp;"Arial"&amp;11Version Date: &lt;DD/MMM/YYYY&gt;&amp;R&amp;"Arial"&amp;10Study Code: &lt;Code&gt;
-System: &lt;System&gt;</ns0:oddHeader>
+&amp;"Arial"&amp;11Version Date: &lt;DD/MMM/YYYY&gt;&amp;R&amp;G</ns0:oddHeader>
     <ns0:oddFooter>&amp;L&amp;"Arial,Standard"GCPS_DMF_012.8_D&amp;C&amp;"Arial,Standard"Effective Date: 16/DEC/2024&amp;R&amp;"Arial,Standard"Page &amp;P of &amp;N</ns0:oddFooter>
   </ns0:headerFooter>
   <ns0:legacyDrawingHF ns4:id="rId2"/>

</xml_diff>